<commit_message>
OK09: tydeligere forutsetninger og tips i 1A
</commit_message>
<xml_diff>
--- a/pensum/ok09/OK09_Budsjettering_Oppgaver_v9.xlsx
+++ b/pensum/ok09/OK09_Budsjettering_Oppgaver_v9.xlsx
@@ -774,10 +774,16 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="105" customHeight="1">
+    <row r="10" ht="215" customHeight="1">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Salgsinntekt 24 000 000 kr: 7,1 % mer enn i 2026, fordi to nye rammeavtaler er signert. Varekostnad: 37,5 % av salget, som i 2026 (8 390 000 / 22 400 000). Lønn: 7 500 000 kr i brutto lønn til alle 18 ansatte etter lønnsoppgjøret (i 2026 var den 10 660 000 / 1,468 = om lag 7 260 000), med 46,8 % sosiale kostnader etter bokas tabell 2.4. Avskrivninger: 620 000 på det bedriften har, pluss termograferingsutstyr til 480 000 kr som kjøpes i mars og avskrives lineært over 4 år, altså 120 000 i året og 10 000 per måned fra og med mars. Andre driftskostnader: 1 500 000 kr, om lag 8 % over fjorårets 1 386 000. Renteinntekter som i fjor, 56 000. Rentekostnad: 7,5 % av banklånet på 2 800 000. Avdraget på lånet er ikke en kostnad.</t>
+          <t>Salgsinntekt: 24 000 000 kr. Det er 7,1 % mer enn i 2026, fordi to nye rammeavtaler er signert. Tallet står ferdig i tabellen.
+Varekostnad: 37,5 % av salget. Hvorfor: i 2026 gikk 8 390 000 av 22 400 000 kr til materiell og innleie, og 8 390 000 / 22 400 000 = 0,375 = 37,5 %. Vi antar at materiellet følger salget også i 2027: mer salg, mer materiell. Regn derfor 37,5 % av årets salg, ikke fjorårets varekostnad pluss noe.
+Lønnskostnad: brutto lønn 7 500 000 kr til alle 18 ansatte etter lønnsoppgjøret, pluss 46,8 % sosiale kostnader (feriepenger, arbeidsgiveravgift, pensjon m.m., bokas tabell 2.4). Lønnskostnad = 7 500 000 × 1,468.
+Avskrivninger: 620 000 kr på det bedriften allerede eier, pluss nytt termograferingsutstyr til 480 000 kr som kjøpes i mars og avskrives over 4 år. Det er 120 000 i året, 10 000 per måned, og i 2027 blir det 10 måneder (mars til desember).
+Andre driftskostnader: 1 500 000 kr, om lag 8 % over fjorårets 1 386 000. Står ferdig i tabellen.
+Renteinntekter: som i fjor, 56 000 kr. Står ferdig i tabellen.
+Rentekostnad: 7,5 % av banklånet på 2 800 000 kr. Avdraget på lånet er ikke en kostnad, for pengene betales tilbake, de brukes ikke opp.</t>
         </is>
       </c>
     </row>
@@ -936,7 +942,7 @@
         </is>
       </c>
       <c r="C27" s="12">
-        <f>IF(D14="","Skriv svaret i den gule cellen.",IF(ISTEXT(D14),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D14-(D13*0.375))&lt;=0.99,"Riktig.",IF(ABS(D14-(D13*0.625))&lt;=0.99,"Du har regnet bruttofortjenesten (62,5 %). Varekostnaden er resten: 37,5 % av salget.",IF(ABS(D14-(8390000*1.071))&lt;=0.99,"Du har økt fjorårets varekostnad med 7,1 %. Det gir nesten det samme, men forutsetningen er 37,5 % av salget på 24 000 000.",IF(IFERROR(AND(D14&lt;&gt;0,(D13*0.375)&lt;&gt;0,ROUND(LOG10(ABS(D14/(D13*0.375))),0)&lt;&gt;0,ABS(LOG10(ABS(D14/(D13*0.375)))-ROUND(LOG10(ABS(D14/(D13*0.375))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D14-(D13*0.375))&lt;=MAX(0.99,0.01*ABS(D13*0.375)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D14&gt;(D13*0.375),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Varekostnad = salgsinntekt × 37,5 %.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Varekostnad = salgsinntekt × 37,5 %."))))))))</f>
+        <f>IF(D14="","Skriv svaret i den gule cellen.",IF(ISTEXT(D14),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D14-(D13*0.375))&lt;=0.99,"Riktig.",IF(ABS(D14-(D13*0.625))&lt;=0.99,"Du har regnet bruttofortjenesten (62,5 %). Varekostnaden er resten: 37,5 % av salget.",IF(ABS(D14-(8390000*1.071))&lt;=0.99,"Du har økt fjorårets varekostnad med 7,1 %. Det gir nesten det samme, men forutsetningen er 37,5 % av salget på 24 000 000.",IF(ABS(D14-(8390000))&lt;=0.99,"Du har fått fjorårets varekostnad. I budsjettet skal du regne 37,5 % av årets salg: skriv =D13*37,5% i den gule cellen.",IF(IFERROR(AND(D14&lt;&gt;0,(D13*0.375)&lt;&gt;0,ROUND(LOG10(ABS(D14/(D13*0.375))),0)&lt;&gt;0,ABS(LOG10(ABS(D14/(D13*0.375)))-ROUND(LOG10(ABS(D14/(D13*0.375))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D14-(D13*0.375))&lt;=MAX(0.99,0.01*ABS(D13*0.375)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D14&gt;(D13*0.375),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Varekostnaden er den delen av salget som går til materiell og innleie: 37,5 %, samme andel som i 2026. Skriv =D13*37,5% (årets salg × 37,5 %).","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Varekostnaden er den delen av salget som går til materiell og innleie: 37,5 %, samme andel som i 2026. Skriv =D13*37,5% (årets salg × 37,5 %).")))))))))</f>
         <v/>
       </c>
     </row>
@@ -947,7 +953,7 @@
         </is>
       </c>
       <c r="C28" s="12">
-        <f>IF(D15="","Skriv svaret i den gule cellen.",IF(ISTEXT(D15),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D15-(7500000*1.468))&lt;=0.99,"Riktig.",IF(ABS(D15-(7500000))&lt;=0.99,"Du har satt inn lønna alene. De sosiale kostnadene på 46,8 % kommer på toppen: gang med 1,468.",IF(ABS(D15-(7500000*0.468))&lt;=0.99,"Du har regnet bare de sosiale kostnadene. Lønnskostnaden er lønna pluss de sosiale: 7 500 000 × 1,468.",IF(ABS(D15-(7500000*1.12*1.141))&lt;=0.99,"Du har tatt bare feriepenger og arbeidsgiveravgift. Boka regner også pensjon, helligdager, forsikring og sykepenger: 46,8 % til sammen.",IF(IFERROR(AND(D15&lt;&gt;0,(7500000*1.468)&lt;&gt;0,ROUND(LOG10(ABS(D15/(7500000*1.468))),0)&lt;&gt;0,ABS(LOG10(ABS(D15/(7500000*1.468)))-ROUND(LOG10(ABS(D15/(7500000*1.468))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D15-(7500000*1.468))&lt;=MAX(0.99,0.01*ABS(7500000*1.468)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D15&gt;(7500000*1.468),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Lønnskostnad = lønn × (1 + 0,468).","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Lønnskostnad = lønn × (1 + 0,468).")))))))))</f>
+        <f>IF(D15="","Skriv svaret i den gule cellen.",IF(ISTEXT(D15),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D15-(7500000*1.468))&lt;=0.99,"Riktig.",IF(ABS(D15-(7500000))&lt;=0.99,"Du har satt inn lønna alene. De sosiale kostnadene på 46,8 % kommer på toppen: gang med 1,468.",IF(ABS(D15-(7500000*0.468))&lt;=0.99,"Du har regnet bare de sosiale kostnadene. Lønnskostnaden er lønna pluss de sosiale: 7 500 000 × 1,468.",IF(ABS(D15-(7500000*1.12*1.141))&lt;=0.99,"Du har tatt bare feriepenger og arbeidsgiveravgift. Boka regner også pensjon, helligdager, forsikring og sykepenger: 46,8 % til sammen.",IF(IFERROR(AND(D15&lt;&gt;0,(7500000*1.468)&lt;&gt;0,ROUND(LOG10(ABS(D15/(7500000*1.468))),0)&lt;&gt;0,ABS(LOG10(ABS(D15/(7500000*1.468)))-ROUND(LOG10(ABS(D15/(7500000*1.468))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D15-(7500000*1.468))&lt;=MAX(0.99,0.01*ABS(7500000*1.468)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D15&gt;(7500000*1.468),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Lønnskostnad = lønna pluss 46,8 % sosiale kostnader. Skriv =7500000*1,468.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Lønnskostnad = lønna pluss 46,8 % sosiale kostnader. Skriv =7500000*1,468.")))))))))</f>
         <v/>
       </c>
     </row>
@@ -958,7 +964,7 @@
         </is>
       </c>
       <c r="C29" s="12">
-        <f>IF(D16="","Skriv svaret i den gule cellen.",IF(ISTEXT(D16),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D16-(620000+480000/4/12*10))&lt;=0.99,"Riktig.",IF(ABS(D16-(620000+480000/4))&lt;=0.99,"Du har tatt et helt år på termograferingsutstyret. Det kjøpes i mars, så det er 10 måneder à 10 000 i 2027.",IF(ABS(D16-(620000))&lt;=0.99,"Du har glemt det nye utstyret. 480 000 over 4 år er 10 000 per måned, fra mars: 100 000 i 2027.",IF(ABS(D16-(620000+480000))&lt;=0.99,"Du har tatt hele kjøpesummen som kostnad. Utstyret avskrives over 4 år; bare 100 000 er kostnad i 2027.",IF(IFERROR(AND(D16&lt;&gt;0,(620000+480000/4/12*10)&lt;&gt;0,ROUND(LOG10(ABS(D16/(620000+480000/4/12*10))),0)&lt;&gt;0,ABS(LOG10(ABS(D16/(620000+480000/4/12*10)))-ROUND(LOG10(ABS(D16/(620000+480000/4/12*10))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D16-(620000+480000/4/12*10))&lt;=MAX(0.99,0.01*ABS(620000+480000/4/12*10)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D16&gt;(620000+480000/4/12*10),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Avskrivninger = 620 000 + 480 000 / 4 år / 12 måneder × 10 måneder.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Avskrivninger = 620 000 + 480 000 / 4 år / 12 måneder × 10 måneder.")))))))))</f>
+        <f>IF(D16="","Skriv svaret i den gule cellen.",IF(ISTEXT(D16),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D16-(620000+480000/4/12*10))&lt;=0.99,"Riktig.",IF(ABS(D16-(620000+480000/4))&lt;=0.99,"Du har tatt et helt år på termograferingsutstyret. Det kjøpes i mars, så det er 10 måneder à 10 000 i 2027.",IF(ABS(D16-(620000))&lt;=0.99,"Du har glemt det nye utstyret. 480 000 over 4 år er 10 000 per måned, fra mars: 100 000 i 2027.",IF(ABS(D16-(620000+480000))&lt;=0.99,"Du har tatt hele kjøpesummen som kostnad. Utstyret avskrives over 4 år; bare 100 000 er kostnad i 2027.",IF(IFERROR(AND(D16&lt;&gt;0,(620000+480000/4/12*10)&lt;&gt;0,ROUND(LOG10(ABS(D16/(620000+480000/4/12*10))),0)&lt;&gt;0,ABS(LOG10(ABS(D16/(620000+480000/4/12*10)))-ROUND(LOG10(ABS(D16/(620000+480000/4/12*10))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D16-(620000+480000/4/12*10))&lt;=MAX(0.99,0.01*ABS(620000+480000/4/12*10)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D16&gt;(620000+480000/4/12*10),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Avskrivninger = det gamle (620 000) pluss det nye utstyret for 10 måneder: 480 000 / 4 år / 12 måneder × 10. Skriv =620000+480000/4/12*10.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Avskrivninger = det gamle (620 000) pluss det nye utstyret for 10 måneder: 480 000 / 4 år / 12 måneder × 10. Skriv =620000+480000/4/12*10.")))))))))</f>
         <v/>
       </c>
     </row>
@@ -969,7 +975,7 @@
         </is>
       </c>
       <c r="C30" s="12">
-        <f>IF(D18="","Skriv svaret i den gule cellen.",IF(ISTEXT(D18),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D18-(D13-D14-D15-D16-D17))&lt;=0.99,"Riktig.",IF(ABS(D18-(D13-D14-D15-D16-D17-210000))&lt;=0.99,"Du har trukket fra rentekostnaden. Den kommer under driftsresultatet, ikke i det.",IF(ABS(D18-(D13-D14-D15-D17))&lt;=0.99,"Du har glemt avskrivningene. De er en kostnad selv om ingen penger går ut i 2027.",IF(IFERROR(AND(D18&lt;&gt;0,(D13-D14-D15-D16-D17)&lt;&gt;0,ROUND(LOG10(ABS(D18/(D13-D14-D15-D16-D17))),0)&lt;&gt;0,ABS(LOG10(ABS(D18/(D13-D14-D15-D16-D17)))-ROUND(LOG10(ABS(D18/(D13-D14-D15-D16-D17))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D18-(D13-D14-D15-D16-D17))&lt;=MAX(0.99,0.01*ABS(D13-D14-D15-D16-D17)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D18&gt;(D13-D14-D15-D16-D17),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Driftsresultat = salgsinntekt − varekostnad − lønnskostnad − avskrivninger − andre driftskostnader.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Driftsresultat = salgsinntekt − varekostnad − lønnskostnad − avskrivninger − andre driftskostnader."))))))))</f>
+        <f>IF(D18="","Skriv svaret i den gule cellen.",IF(ISTEXT(D18),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D18-(D13-D14-D15-D16-D17))&lt;=0.99,"Riktig.",IF(ABS(D18-(D13-D14-D15-D16-D17-210000))&lt;=0.99,"Du har trukket fra rentekostnaden. Den kommer under driftsresultatet, ikke i det.",IF(ABS(D18-(D13-D14-D15-D17))&lt;=0.99,"Du har glemt avskrivningene. De er en kostnad selv om ingen penger går ut i 2027.",IF(IFERROR(AND(D18&lt;&gt;0,(D13-D14-D15-D16-D17)&lt;&gt;0,ROUND(LOG10(ABS(D18/(D13-D14-D15-D16-D17))),0)&lt;&gt;0,ABS(LOG10(ABS(D18/(D13-D14-D15-D16-D17)))-ROUND(LOG10(ABS(D18/(D13-D14-D15-D16-D17))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D18-(D13-D14-D15-D16-D17))&lt;=MAX(0.99,0.01*ABS(D13-D14-D15-D16-D17)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D18&gt;(D13-D14-D15-D16-D17),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Driftsresultat = salgsinntekt minus alle driftskostnadene. Skriv =D13-D14-D15-D16-D17.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Driftsresultat = salgsinntekt minus alle driftskostnadene. Skriv =D13-D14-D15-D16-D17."))))))))</f>
         <v/>
       </c>
     </row>
@@ -980,7 +986,7 @@
         </is>
       </c>
       <c r="C31" s="12">
-        <f>IF(D20="","Skriv svaret i den gule cellen.",IF(ISTEXT(D20),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D20-(2800000*0.075))&lt;=0.99,"Riktig.",IF(ABS(D20-(2800000*0.075+560000))&lt;=0.99,"Du har lagt til avdraget på 560 000. Avdrag er ikke en kostnad; bare renten er det.",IF(ABS(D20-(232500))&lt;=0.99,"Du har tatt fjorårets rentekostnad. Forutsetningen er 7,5 % av banklånet på 2 800 000.",IF(IFERROR(AND(D20&lt;&gt;0,(2800000*0.075)&lt;&gt;0,ROUND(LOG10(ABS(D20/(2800000*0.075))),0)&lt;&gt;0,ABS(LOG10(ABS(D20/(2800000*0.075)))-ROUND(LOG10(ABS(D20/(2800000*0.075))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D20-(2800000*0.075))&lt;=MAX(0.99,0.01*ABS(2800000*0.075)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D20&gt;(2800000*0.075),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Rentekostnad = 2 800 000 × 7,5 %.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Rentekostnad = 2 800 000 × 7,5 %."))))))))</f>
+        <f>IF(D20="","Skriv svaret i den gule cellen.",IF(ISTEXT(D20),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D20-(2800000*0.075))&lt;=0.99,"Riktig.",IF(ABS(D20-(2800000*0.075+560000))&lt;=0.99,"Du har lagt til avdraget på 560 000. Avdrag er ikke en kostnad; bare renten er det.",IF(ABS(D20-(232500))&lt;=0.99,"Du har tatt fjorårets rentekostnad. Forutsetningen er 7,5 % av banklånet på 2 800 000.",IF(IFERROR(AND(D20&lt;&gt;0,(2800000*0.075)&lt;&gt;0,ROUND(LOG10(ABS(D20/(2800000*0.075))),0)&lt;&gt;0,ABS(LOG10(ABS(D20/(2800000*0.075)))-ROUND(LOG10(ABS(D20/(2800000*0.075))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D20-(2800000*0.075))&lt;=MAX(0.99,0.01*ABS(2800000*0.075)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D20&gt;(2800000*0.075),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Rentekostnad = banklånet × renten. Skriv =2800000*7,5%.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Rentekostnad = banklånet × renten. Skriv =2800000*7,5%."))))))))</f>
         <v/>
       </c>
     </row>
@@ -991,7 +997,7 @@
         </is>
       </c>
       <c r="C32" s="12">
-        <f>IF(D21="","Skriv svaret i den gule cellen.",IF(ISTEXT(D21),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D21-(D18+D19-D20))&lt;=0.99,"Riktig.",IF(ABS(D21-(D18-D20))&lt;=0.99,"Du har glemt renteinntektene på 56 000.",IF(ABS(D21-(D18-D19-D20))&lt;=0.99,"Renteinntektene skal legges til, ikke trekkes fra.",IF(IFERROR(AND(D21&lt;&gt;0,(D18+D19-D20)&lt;&gt;0,ROUND(LOG10(ABS(D21/(D18+D19-D20))),0)&lt;&gt;0,ABS(LOG10(ABS(D21/(D18+D19-D20)))-ROUND(LOG10(ABS(D21/(D18+D19-D20))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D21-(D18+D19-D20))&lt;=MAX(0.99,0.01*ABS(D18+D19-D20)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D21&gt;(D18+D19-D20),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Resultat før skatt = driftsresultat + renteinntekter − rentekostnader.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Resultat før skatt = driftsresultat + renteinntekter − rentekostnader."))))))))</f>
+        <f>IF(D21="","Skriv svaret i den gule cellen.",IF(ISTEXT(D21),"Skriv bare tallet, uten mellomrom, enhet eller tekst. Enheten står ved siden av cellen. Du kan også skrive regnestykket med likhetstegn foran, for eksempel =2100000/7300.",IF(ABS(D21-(D18+D19-D20))&lt;=0.99,"Riktig.",IF(ABS(D21-(D18-D20))&lt;=0.99,"Du har glemt renteinntektene på 56 000.",IF(ABS(D21-(D18-D19-D20))&lt;=0.99,"Renteinntektene skal legges til, ikke trekkes fra.",IF(IFERROR(AND(D21&lt;&gt;0,(D18+D19-D20)&lt;&gt;0,ROUND(LOG10(ABS(D21/(D18+D19-D20))),0)&lt;&gt;0,ABS(LOG10(ABS(D21/(D18+D19-D20)))-ROUND(LOG10(ABS(D21/(D18+D19-D20))),0))&lt;0.004),FALSE),"Sifrene stemmer, men antall nuller eller plasseringen av kommaet er feil. Sjekk om du har regnet i kroner, tusen kroner eller prosent.",IF(ABS(D21-(D18+D19-D20))&lt;=MAX(0.99,0.01*ABS(D18+D19-D20)),"Riktig. Svaret ditt ligger litt fra arkets tall fordi du har rundet av underveis. Det er helt greit.",IF(D21&gt;(D18+D19-D20),"Ikke riktig ennå. Svaret ditt er for høyt. Tips: Resultat før skatt = driftsresultat pluss renteinntekter minus rentekostnader. Skriv =D18+D19-D20.","Ikke riktig ennå. Svaret ditt er for lavt. Tips: Resultat før skatt = driftsresultat pluss renteinntekter minus rentekostnader. Skriv =D18+D19-D20."))))))))</f>
         <v/>
       </c>
     </row>

</xml_diff>